<commit_message>
fix(template): WhatIf sheet ships with key/value header row
</commit_message>
<xml_diff>
--- a/templates/workbook_template.xlsx
+++ b/templates/workbook_template.xlsx
@@ -1135,72 +1135,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="004472C4"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>shareholder_name</t>
+          <t>key</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>black_voting_rights_pct</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>black_economic_interest_pct</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>black_women_voting_rights_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>black_women_economic_interest_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>black_designated_groups_pct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>net_value_pct</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>new_entrants_pct</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>effective_date</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>evidence_id</t>
+          <t>value</t>
         </is>
       </c>
     </row>
@@ -1209,85 +1155,65 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>employee_id</t>
+          <t>shareholder_name</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>black_voting_rights_pct</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>race</t>
+          <t>black_economic_interest_pct</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>is_black</t>
+          <t>black_women_voting_rights_pct</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>black_women_economic_interest_pct</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>black_designated_groups_pct</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>foreign_national</t>
+          <t>net_value_pct</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>occupational_level</t>
+          <t>new_entrants_pct</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>is_executive_director</t>
+          <t>effective_date</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>is_non_executive_director</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>start_date</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>end_date</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>fte_months_in_period</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>annual_salary</t>
+          <t>evidence_id</t>
         </is>
       </c>
     </row>
@@ -1296,89 +1222,85 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="0000B050"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>employee_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>employee_id</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>course_name</t>
+          <t>race</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>training_category</t>
+          <t>is_black</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>accredited</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>training_spend</t>
+          <t>disability</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>salary_cost_during_training</t>
+          <t>foreign_national</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>occupational_level</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>is_executive_director</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>is_non_executive_director</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>is_discretionary</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>evidence_id</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>fte_months_in_period</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>annual_salary</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1309,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0000B050"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
@@ -1400,57 +1336,57 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>participant_id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>is_employee</t>
+          <t>employee_id</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>race</t>
+          <t>course_name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>training_category</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>disability</t>
+          <t>accredited</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>learnership_type</t>
+          <t>training_spend</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>saqa_registered</t>
+          <t>salary_cost_during_training</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>stipend_paid</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>absorbed</t>
+          <t>is_discretionary</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -1464,58 +1400,73 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>beneficiary_id</t>
+          <t>participant_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>is_employee</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>race</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>disability</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>institution</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>internal_or_external</t>
+          <t>learnership_type</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>academic_year</t>
+          <t>saqa_registered</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>start_date</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>stipend_paid</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>absorbed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>evidence_id</t>
         </is>
@@ -1524,4 +1475,66 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="004472C4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>beneficiary_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>disability</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>institution</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>internal_or_external</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>academic_year</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>